<commit_message>
40 pin connector reposition
</commit_message>
<xml_diff>
--- a/Project Outputs for de10ext/bom.xlsx
+++ b/Project Outputs for de10ext/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\xmoshte\projects\de10ext\hardware\de10ext\Project Outputs for de10ext\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47047578-053C-435E-BC45-69D63ECB8EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64CE838F-8398-42E9-AC84-9AAE2ADFB03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{3F3C5F57-A3A6-4BDD-A238-42EEE3BDA570}"/>
   </bookViews>
@@ -42,20 +42,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="136">
   <si>
     <t>KLPX-0848A-2-W</t>
   </si>
   <si>
-    <t>AJ 1</t>
-  </si>
-  <si>
     <t>KLPX-0848A-2-R</t>
   </si>
   <si>
-    <t>AJ 2</t>
-  </si>
-  <si>
     <t>100n 50V</t>
   </si>
   <si>
@@ -122,9 +116,6 @@
     <t>FB1</t>
   </si>
   <si>
-    <t>USB1046-GF</t>
-  </si>
-  <si>
     <t>USB-A (USB TYPE-A) USB 2.0 Receptacle Connector 4 Position Surface Mount, Through Hole</t>
   </si>
   <si>
@@ -212,9 +203,6 @@
     <t>U1</t>
   </si>
   <si>
-    <t>2223</t>
-  </si>
-  <si>
     <t>U2</t>
   </si>
   <si>
@@ -453,6 +441,15 @@
   </si>
   <si>
     <t>600Ω@100MHz 1 Line Ferrite Bead 0603 500mA 380mΩ</t>
+  </si>
+  <si>
+    <t>AJ1</t>
+  </si>
+  <si>
+    <t>AJ2</t>
+  </si>
+  <si>
+    <t>DNP</t>
   </si>
 </sst>
 </file>
@@ -506,13 +503,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="4" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="-0.249977111117893"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -556,13 +553,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -571,14 +565,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -920,638 +919,638 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="18.81640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" style="7" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" style="6" customWidth="1"/>
     <col min="5" max="6" width="18.81640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="111.6328125" style="2" customWidth="1"/>
     <col min="8" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D1" s="10"/>
-    </row>
-    <row r="2" spans="1:7" s="4" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="5" t="s">
+    <row r="1" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D1" s="8"/>
+    </row>
+    <row r="2" spans="1:7" s="3" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D3" s="11">
+        <v>1</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" s="11">
+        <v>1</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G2" s="5" t="s">
+      <c r="F4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="7">
-        <v>1</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D4" s="8">
-        <v>1</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D5" s="7">
+        <v>3</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="6">
         <v>13</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D6" s="7">
+        <v>5</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="6">
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="7">
+        <v>120</v>
+      </c>
+      <c r="D7" s="6">
         <v>4</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D8" s="7">
+        <v>11</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" s="6">
         <v>2</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D9" s="7">
+        <v>122</v>
+      </c>
+      <c r="D9" s="6">
         <v>1</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D10" s="7">
+        <v>122</v>
+      </c>
+      <c r="D10" s="6">
         <v>1</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="C11" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D11" s="7">
+        <v>124</v>
+      </c>
+      <c r="D11" s="6">
         <v>1</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="C12" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D12" s="7">
+        <v>125</v>
+      </c>
+      <c r="D12" s="6">
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D14" s="11">
+        <v>5</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D13" s="7">
-        <v>1</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D14" s="7">
-        <v>5</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D15" s="7">
+        <v>127</v>
+      </c>
+      <c r="D15" s="6">
         <v>1</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D16" s="7">
+        <v>126</v>
+      </c>
+      <c r="D16" s="6">
         <v>1</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D17" s="7">
+        <v>128</v>
+      </c>
+      <c r="D17" s="6">
         <v>1</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="D18" s="7">
+        <v>129</v>
+      </c>
+      <c r="D18" s="6">
         <v>1</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D19" s="7">
+        <v>122</v>
+      </c>
+      <c r="D19" s="6">
         <v>2</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D20" s="7">
+        <v>123</v>
+      </c>
+      <c r="D20" s="6">
         <v>2</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D21" s="7">
+        <v>122</v>
+      </c>
+      <c r="D21" s="6">
         <v>2</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D22" s="7">
+        <v>122</v>
+      </c>
+      <c r="D22" s="6">
         <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D23" s="7">
+        <v>122</v>
+      </c>
+      <c r="D23" s="6">
         <v>15</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D24" s="7">
+        <v>122</v>
+      </c>
+      <c r="D24" s="6">
         <v>12</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D25" s="7">
+        <v>122</v>
+      </c>
+      <c r="D25" s="6">
         <v>2</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D26" s="6">
+        <v>1</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D26" s="7">
+      <c r="C27" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D27" s="11">
         <v>1</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D27" s="7">
-        <v>1</v>
-      </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" s="13">
+        <v>2223</v>
+      </c>
+      <c r="G27" s="10" t="s">
         <v>112</v>
-      </c>
-      <c r="F27" s="3">
-        <v>2223</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="D28" s="7">
+        <v>131</v>
+      </c>
+      <c r="D28" s="6">
         <v>1</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D29" s="10"/>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D29" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>